<commit_message>
Adjusted code to excel source
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kgafe\Desktop\NMS Upgrade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FB26E91-571A-4C9C-BCB8-269366A57B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7CD148-4B59-41D6-83E5-55C9CD7BACC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>SERIAL</t>
   </si>
@@ -94,6 +94,15 @@
   </si>
   <si>
     <t>TEMP</t>
+  </si>
+  <si>
+    <t>4GW00805</t>
+  </si>
+  <si>
+    <t>KISSAMOS</t>
+  </si>
+  <si>
+    <t>21/01/2026 10:00</t>
   </si>
 </sst>
 </file>
@@ -101,7 +110,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="m/d/yy\ h:mm;@"/>
+    <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -132,9 +141,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -415,9 +429,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -653,6 +669,35 @@
         <v>40</v>
       </c>
     </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>-98</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>